<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client · 43 sel berubah · Barang Keluar , Barang Masuk, ... · update penggunaan reagent dan stock yang tersedia
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F60032A-4B84-4699-8631-CBAB5797089E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AF07B3-0C8B-46E0-8059-E9A79EC6108B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Stock Barang" sheetId="1" r:id="rId1"/>
     <sheet name="Barang Masuk" sheetId="2" r:id="rId2"/>
-    <sheet name="Barang Keluar " sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
+    <sheet name="Barang Keluar " sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -388,36 +388,6 @@
   </cellStyles>
   <dxfs count="15">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -602,6 +572,13 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -624,13 +601,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -667,6 +637,36 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -687,22 +687,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
   <autoFilter ref="B3:H21" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}"/>
   <tableColumns count="7">
-    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="3">
       <calculatedColumnFormula>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="5">
+    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="2">
       <calculatedColumnFormula>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="4">
+    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="1">
       <calculatedColumnFormula>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1134,11 +1134,11 @@
       </c>
       <c r="F5" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="G5" s="13">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>33</v>
@@ -1152,7 +1152,7 @@
         <v>13</v>
       </c>
       <c r="D6" s="2">
-        <v>5900</v>
+        <v>5750</v>
       </c>
       <c r="E6" s="2">
         <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
@@ -1160,11 +1160,11 @@
       </c>
       <c r="F6" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>1500</v>
+        <v>2375</v>
       </c>
       <c r="G6" s="13">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>4400</v>
+        <v>3375</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>33</v>
@@ -1182,15 +1182,15 @@
       </c>
       <c r="E7" s="2">
         <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="F7" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>2250</v>
+        <v>3500</v>
       </c>
       <c r="G7" s="13">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>5250</v>
+        <v>9000</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>33</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="F12" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G12" s="14">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>6375</v>
+        <v>6325</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>33</v>
@@ -1493,15 +1493,15 @@
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>3999</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G10">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="lessThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1545,13 +1545,19 @@
       <c r="B5" s="8">
         <v>1</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="7"/>
+      <c r="C5" s="9">
+        <v>46277</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="E5" s="7" t="str">
         <f>IFERROR(VLOOKUP(D5,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F5" s="7"/>
+        <v>Kapur</v>
+      </c>
+      <c r="F5" s="7">
+        <v>5000</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="8">
@@ -4610,6 +4616,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684DB87B-F02C-41BA-A196-5B8F96176BFB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C4F271-B1B8-49EF-AE8E-5ADDB846D57A}">
   <dimension ref="B4:K315"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4925,7 +4940,7 @@
         <v>Kapur</v>
       </c>
       <c r="F17" s="7">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="G17" t="s">
         <v>25</v>
@@ -4998,13 +5013,19 @@
       <c r="B21" s="8">
         <v>17</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
+      <c r="C21" s="9">
+        <v>46276</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>8</v>
+      </c>
       <c r="E21" s="7" t="str">
         <f>IFERROR(VLOOKUP(D21,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="7"/>
+        <v>Sandios</v>
+      </c>
+      <c r="F21" s="7">
+        <v>375</v>
+      </c>
       <c r="G21" t="s">
         <v>25</v>
       </c>
@@ -5013,13 +5034,19 @@
       <c r="B22" s="8">
         <v>18</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="C22" s="9">
+        <v>46277</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>8</v>
+      </c>
       <c r="E22" s="7" t="str">
         <f>IFERROR(VLOOKUP(D22,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="7"/>
+        <v>Sandios</v>
+      </c>
+      <c r="F22" s="7">
+        <v>125</v>
+      </c>
       <c r="G22" t="s">
         <v>25</v>
       </c>
@@ -5028,13 +5055,19 @@
       <c r="B23" s="8">
         <v>19</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
+      <c r="C23" s="9">
+        <v>46278</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>8</v>
+      </c>
       <c r="E23" s="7" t="str">
         <f>IFERROR(VLOOKUP(D23,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="7"/>
+        <v>Sandios</v>
+      </c>
+      <c r="F23" s="7">
+        <v>375</v>
+      </c>
       <c r="G23" t="s">
         <v>25</v>
       </c>
@@ -5043,13 +5076,19 @@
       <c r="B24" s="8">
         <v>20</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
+      <c r="C24" s="9">
+        <v>46277</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="E24" s="7" t="str">
         <f>IFERROR(VLOOKUP(D24,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F24" s="7"/>
+        <v>Carbon</v>
+      </c>
+      <c r="F24" s="7">
+        <v>500</v>
+      </c>
       <c r="G24" t="s">
         <v>25</v>
       </c>
@@ -5058,13 +5097,19 @@
       <c r="B25" s="8">
         <v>21</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
+      <c r="C25" s="9">
+        <v>46276</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="E25" s="7" t="str">
         <f>IFERROR(VLOOKUP(D25,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="7"/>
+        <v>Floculant</v>
+      </c>
+      <c r="F25" s="7">
+        <v>50</v>
+      </c>
       <c r="G25" t="s">
         <v>25</v>
       </c>
@@ -5073,13 +5118,19 @@
       <c r="B26" s="8">
         <v>22</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
+      <c r="C26" s="9">
+        <v>46267</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="E26" s="7" t="str">
         <f>IFERROR(VLOOKUP(D26,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="7"/>
+        <v>Kapur</v>
+      </c>
+      <c r="F26" s="7">
+        <v>500</v>
+      </c>
       <c r="G26" t="s">
         <v>25</v>
       </c>
@@ -5088,13 +5139,19 @@
       <c r="B27" s="8">
         <v>23</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
+      <c r="C27" s="9">
+        <v>46268</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="E27" s="7" t="str">
         <f>IFERROR(VLOOKUP(D27,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="7"/>
+        <v>Kapur</v>
+      </c>
+      <c r="F27" s="7">
+        <v>250</v>
+      </c>
       <c r="G27" t="s">
         <v>25</v>
       </c>
@@ -7738,13 +7795,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684DB87B-F02C-41BA-A196-5B8F96176BFB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client · tidak ada perubahan isi
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -388,6 +388,36 @@
   </cellStyles>
   <dxfs count="15">
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -572,13 +602,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -601,6 +624,13 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -637,36 +667,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -687,22 +687,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
   <autoFilter ref="B3:H21" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}"/>
   <tableColumns count="7">
-    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="3">
+    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="6">
       <calculatedColumnFormula>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="5">
       <calculatedColumnFormula>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="4">
       <calculatedColumnFormula>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1493,15 +1493,15 @@
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>3999</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G10">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client · 6 sel berubah · Barang Keluar , Stock Barang
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AF07B3-0C8B-46E0-8059-E9A79EC6108B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702BA5E7-3C29-4EE4-A6C3-5D30D134DF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
   </bookViews>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="F12" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="G12" s="14">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>6325</v>
+        <v>6300</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>33</v>
@@ -5160,13 +5160,19 @@
       <c r="B28" s="8">
         <v>24</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
+      <c r="C28" s="9">
+        <v>46269</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="E28" s="7" t="str">
         <f>IFERROR(VLOOKUP(D28,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F28" s="7"/>
+        <v>Floculant</v>
+      </c>
+      <c r="F28" s="7">
+        <v>25</v>
+      </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client · 12 sel berubah · Barang Masuk, Stock Barang
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC2ADA7-55B6-4A5C-80AD-B0C43FB76B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35211DD-B11A-41BB-BA0B-30515A939761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Barang Masuk" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId2"/>
-    <sheet name="Stock Barang" sheetId="1" r:id="rId3"/>
-    <sheet name="Barang Keluar " sheetId="3" r:id="rId4"/>
+    <sheet name="Stock Barang" sheetId="1" r:id="rId1"/>
+    <sheet name="Barang Masuk" sheetId="2" r:id="rId2"/>
+    <sheet name="Barang Keluar " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -93,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -388,62 +387,6 @@
   </cellStyles>
   <dxfs count="15">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -490,6 +433,32 @@
         <horizontal style="thin">
           <color indexed="64"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -602,6 +571,13 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -624,13 +600,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -667,6 +636,36 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -687,22 +686,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
   <autoFilter ref="B3:H21" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}"/>
   <tableColumns count="7">
-    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="3">
       <calculatedColumnFormula>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="2">
       <calculatedColumnFormula>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="5">
+    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="1">
       <calculatedColumnFormula>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1044,6 +1043,476 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CAC8830-268B-489B-9A12-01936A5CA5A2}">
+  <dimension ref="B1:H21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="10" customWidth="1"/>
+    <col min="8" max="8" width="15" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="B1" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2">
+        <v>150</v>
+      </c>
+      <c r="E4" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>150</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E5" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>3000</v>
+      </c>
+      <c r="G5" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>2000</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5750</v>
+      </c>
+      <c r="E6" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>3725</v>
+      </c>
+      <c r="G6" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>2025</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2">
+        <v>7500</v>
+      </c>
+      <c r="E7" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>5000</v>
+      </c>
+      <c r="F7" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>3000</v>
+      </c>
+      <c r="G7" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>9500</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2">
+        <v>400</v>
+      </c>
+      <c r="E8" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>250</v>
+      </c>
+      <c r="F8" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>650</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="2">
+        <v>125</v>
+      </c>
+      <c r="E10" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>375</v>
+      </c>
+      <c r="F10" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>500</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="2">
+        <v>14975</v>
+      </c>
+      <c r="E11" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>14975</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="2">
+        <v>6425</v>
+      </c>
+      <c r="E12" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>200</v>
+      </c>
+      <c r="G12" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>6225</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="2">
+        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="2">
+        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="15">
+        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+      <formula>3999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G10">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E498DA0C-37B1-4354-B038-CA23BB50DFD0}">
   <dimension ref="B4:F334"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1093,25 +1562,37 @@
       <c r="B6" s="8">
         <v>2</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="7"/>
+      <c r="C6" s="9">
+        <v>46285</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="E6" s="7" t="str">
         <f>IFERROR(VLOOKUP(D6,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F6" s="7"/>
+        <v>HCL</v>
+      </c>
+      <c r="F6" s="7">
+        <v>375</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="8">
         <v>3</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+      <c r="C7" s="9">
+        <v>46285</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>10</v>
+      </c>
       <c r="E7" s="7" t="str">
         <f>IFERROR(VLOOKUP(D7,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="7"/>
+        <v>Kaustik</v>
+      </c>
+      <c r="F7" s="7">
+        <v>250</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="8">
@@ -4145,486 +4626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684DB87B-F02C-41BA-A196-5B8F96176BFB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CAC8830-268B-489B-9A12-01936A5CA5A2}">
-  <dimension ref="B1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="15" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B1" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2">
-        <v>150</v>
-      </c>
-      <c r="E4" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>150</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2">
-        <v>5000</v>
-      </c>
-      <c r="E5" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>3000</v>
-      </c>
-      <c r="G5" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>2000</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2">
-        <v>5750</v>
-      </c>
-      <c r="E6" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>3725</v>
-      </c>
-      <c r="G6" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>2025</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="2">
-        <v>7500</v>
-      </c>
-      <c r="E7" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>5000</v>
-      </c>
-      <c r="F7" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>3000</v>
-      </c>
-      <c r="G7" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>9500</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="2">
-        <v>400</v>
-      </c>
-      <c r="E8" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>400</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0</v>
-      </c>
-      <c r="E9" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="2">
-        <v>125</v>
-      </c>
-      <c r="E10" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>125</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="2">
-        <v>14975</v>
-      </c>
-      <c r="E11" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>14975</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2">
-        <v>6425</v>
-      </c>
-      <c r="E12" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>200</v>
-      </c>
-      <c r="G12" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>6225</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="12"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="12"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="12"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="12"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G20" s="14">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="12"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="2">
-        <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="2">
-        <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="15">
-        <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="12"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:G1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
-      <formula>3999</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G10">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
-      <formula>500</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
-      <formula>500</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C4F271-B1B8-49EF-AE8E-5ADDB846D57A}">
   <dimension ref="B4:K315"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client · 6 sel berubah · Barang Masuk, Stock Barang
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35211DD-B11A-41BB-BA0B-30515A939761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B829621C-2FE0-4F79-B544-DA30452CAFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
   </bookViews>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -387,6 +387,36 @@
   </cellStyles>
   <dxfs count="15">
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -571,13 +601,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -600,6 +623,13 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -636,36 +666,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -686,22 +686,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}" name="Table1" displayName="Table1" ref="B3:H21" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
   <autoFilter ref="B3:H21" xr:uid="{1AC36863-5F67-4496-A2C7-808F86C284A1}"/>
   <tableColumns count="7">
-    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="3">
+    <tableColumn id="2" xr3:uid="{E78837C8-954C-440F-BCB4-114AA4EBC159}" name="Kode Barang" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{BB8DB245-EB50-4D84-9B3E-D2CF46896708}" name="Nama Barang" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{36BAEBBD-D2E7-42F0-B8AF-873903FEFEA9}" name="Stok Awal " dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{3DA331B5-0C1B-4517-AC2B-660041411D0B}" name="Barang Masuk" dataDxfId="6">
       <calculatedColumnFormula>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{4231B6CF-326F-44B2-8A60-3DCCDB55861D}" name="Barang Keluar " dataDxfId="5">
       <calculatedColumnFormula>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{9472852C-4AF5-44FD-A6F5-E9EDEDD511AE}" name="Stock Akhir" dataDxfId="4">
       <calculatedColumnFormula>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{C780F2FB-0F97-426F-AC7D-196550D5A9CF}" name="Satuan" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E6" s="2">
         <f>SUMIF('Barang Masuk'!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Masuk'!$F$5:$F$29)</f>
-        <v>0</v>
+        <v>6250</v>
       </c>
       <c r="F6" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$315,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$315)</f>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G6" s="13">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>2025</v>
+        <v>8275</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>33</v>
@@ -1492,15 +1492,15 @@
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>3999</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G10">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1598,13 +1598,19 @@
       <c r="B8" s="8">
         <v>4</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+      <c r="C8" s="9">
+        <v>46280</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>8</v>
+      </c>
       <c r="E8" s="7" t="str">
         <f>IFERROR(VLOOKUP(D8,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="7"/>
+        <v>Sandios</v>
+      </c>
+      <c r="F8" s="7">
+        <v>6250</v>
+      </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="8">

</xml_diff>